<commit_message>
update "goi y" and template
</commit_message>
<xml_diff>
--- a/kho_cau_hoi.xlsx
+++ b/kho_cau_hoi.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngovi\OneDrive\Máy tính\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngovi\OneDrive\Máy tính\streamlit-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0441D95A-6954-455A-B22B-5328DD7CAB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC76E663-4BEF-446F-BC2F-59BA3727B728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,18 +16,18 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="dieu_12" localSheetId="0">Sheet1!$A$3</definedName>
-    <definedName name="dieu_133" localSheetId="0">Sheet1!$A$13</definedName>
-    <definedName name="dieu_136" localSheetId="0">Sheet1!$A$14</definedName>
-    <definedName name="dieu_174" localSheetId="0">Sheet1!$A$15</definedName>
-    <definedName name="dieu_188" localSheetId="0">Sheet1!$A$16</definedName>
-    <definedName name="dieu_201" localSheetId="0">Sheet1!$A$17</definedName>
-    <definedName name="dieu_5" localSheetId="0">Sheet1!$A$2</definedName>
-    <definedName name="dieu_79" localSheetId="0">Sheet1!$A$6</definedName>
-    <definedName name="dieu_80" localSheetId="0">Sheet1!$A$7</definedName>
-    <definedName name="dieu_81" localSheetId="0">Sheet1!$A$8</definedName>
-    <definedName name="dieu_82" localSheetId="0">Sheet1!$A$10</definedName>
-    <definedName name="dieu_99" localSheetId="0">Sheet1!$A$12</definedName>
+    <definedName name="dieu_12" localSheetId="0">Sheet1!$B$3</definedName>
+    <definedName name="dieu_133" localSheetId="0">Sheet1!$B$12</definedName>
+    <definedName name="dieu_136" localSheetId="0">Sheet1!$B$13</definedName>
+    <definedName name="dieu_174" localSheetId="0">Sheet1!$B$14</definedName>
+    <definedName name="dieu_188" localSheetId="0">Sheet1!$B$15</definedName>
+    <definedName name="dieu_201" localSheetId="0">Sheet1!$B$16</definedName>
+    <definedName name="dieu_5" localSheetId="0">Sheet1!$B$2</definedName>
+    <definedName name="dieu_79" localSheetId="0">Sheet1!$B$6</definedName>
+    <definedName name="dieu_80" localSheetId="0">Sheet1!$B$7</definedName>
+    <definedName name="dieu_81" localSheetId="0">Sheet1!$B$8</definedName>
+    <definedName name="dieu_82" localSheetId="0">Sheet1!$B$9</definedName>
+    <definedName name="dieu_99" localSheetId="0">Sheet1!$B$11</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
   <si>
     <t>Câu hỏi</t>
   </si>
@@ -268,6 +268,15 @@
 a) Qua kiểm tra phát hiện mạch bảo vệ chính của máy biến áp tác động là do hư hỏng trong mạch bảo vệ và hư hỏng đó đã được khắc phục;
 b) Qua kiểm tra phát hiện mạch bảo vệ chính của máy biến áp tác động là do hư hỏng thiết bị trong vùng bảo vệ chính (nhưng không phải là máy biến áp) và hư hỏng đó đã được khắc phục;
 c) Qua kiểm tra mạch bảo vệ chính, các thiết bị trong vùng bảo vệ chính và không phát hiện hư hỏng, Đơn vị quản lý vận hành đã thực hiện theo quy định tại khoản 2 Điều này</t>
+  </si>
+  <si>
+    <t>STT</t>
+  </si>
+  <si>
+    <t>Gợi ý</t>
+  </si>
+  <si>
+    <t>abcd</t>
   </si>
 </sst>
 </file>
@@ -601,139 +610,235 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.0625" customWidth="1"/>
-    <col min="2" max="2" width="53.625" customWidth="1"/>
+    <col min="2" max="2" width="34.0625" customWidth="1"/>
+    <col min="3" max="3" width="53.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="365.25" x14ac:dyDescent="0.45">
-      <c r="A2" s="1" t="s">
+      <c r="D1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="365.25" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="216" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="216" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="202.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="202.5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="338.25" x14ac:dyDescent="0.45">
-      <c r="A5" s="1" t="s">
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="338.25" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="409.6" x14ac:dyDescent="0.45">
-      <c r="A6" s="1" t="s">
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="270" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="270" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="409.6" x14ac:dyDescent="0.45">
-      <c r="A8" s="1" t="s">
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="365.25" x14ac:dyDescent="0.45">
-      <c r="A10" s="1" t="s">
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="365.25" x14ac:dyDescent="0.45">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="243.75" x14ac:dyDescent="0.45">
-      <c r="A11" s="1" t="s">
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="243.75" x14ac:dyDescent="0.45">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="216.75" x14ac:dyDescent="0.45">
-      <c r="A12" s="1" t="s">
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="216.75" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="409.6" x14ac:dyDescent="0.45">
-      <c r="A13" s="1" t="s">
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="365.25" x14ac:dyDescent="0.45">
-      <c r="A14" s="1" t="s">
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="365.25" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" ht="409.6" x14ac:dyDescent="0.45">
-      <c r="A15" s="1" t="s">
+      <c r="D13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="409.6" x14ac:dyDescent="0.45">
-      <c r="A16" s="1" t="s">
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="409.6" x14ac:dyDescent="0.45">
-      <c r="A17" s="1" t="s">
+      <c r="D15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>31</v>
+      </c>
+      <c r="D16" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update data with "gợi ý"
</commit_message>
<xml_diff>
--- a/kho_cau_hoi.xlsx
+++ b/kho_cau_hoi.xlsx
@@ -1,26 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngovi\OneDrive\Máy tính\streamlit-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27FF4C2-D084-4034-9EE7-86F6710BCBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01218DE0-7E54-469E-8990-2C3D81EA91AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kho câu hỏi" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>STT</t>
   </si>
@@ -258,6 +269,19 @@
 a) Qua kiểm tra phát hiện mạch bảo vệ chính của máy biến áp tác động là do hư hỏng trong mạch bảo vệ và hư hỏng đó đã được khắc phục;
 b) Qua kiểm tra phát hiện mạch bảo vệ chính của máy biến áp tác động là do hư hỏng thiết bị trong vùng bảo vệ chính (nhưng không phải là máy biến áp) và hư hỏng đó đã được khắc phục;
 c) Qua kiểm tra mạch bảo vệ chính, các thiết bị trong vùng bảo vệ chính và không phát hiện hư hỏng, Đơn vị quản lý vận hành đã thực hiện theo quy định tại khoản 2 Điều này</t>
+  </si>
+  <si>
+    <t>Báo cáo cắt điện theo hướng chuẩn: 
+B- Thông báo, c - cho phép, c - chỉnh, đ - đổi, t - thao tác, h- hạn chế, c- chuẩn y</t>
+  </si>
+  <si>
+    <t>Nguyên tắc quyền điều khiển =&gt; Nguyên tắc quyền kiểm tra =&gt; Ủy quyền đk =&gt; Trách nhiệm phân cấp =&gt; Chi tiết phân cấp</t>
+  </si>
+  <si>
+    <t>Tần số; Điện áp, Lưới điện, công suất, phụ tải</t>
+  </si>
+  <si>
+    <t>Hình thức =&gt; Về Lệnh =&gt; Về Người =&gt; Về kênh thông tin</t>
   </si>
 </sst>
 </file>
@@ -527,7 +551,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="148.5">
@@ -541,7 +565,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="162">
@@ -555,7 +579,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="229.5">
@@ -569,7 +593,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="337.5">
@@ -582,9 +606,7 @@
       <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" ht="202.5">
       <c r="A7">
@@ -716,7 +738,7 @@
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C16" s="2" t="s">

</xml_diff>